<commit_message>
Updated the eda file and created the sythentic target feature: nutrient vector containing amounts of magnesium, fibre and polyunsaturated fat (PUFA) instead of omega 3 because the nutrition dataset I am using does not explicitly cite omega 3 it cites polyunsaturated fat. Omega 3 is a main component of PUFAs.
</commit_message>
<xml_diff>
--- a/pcos_data_with_nutrition.xlsx
+++ b/pcos_data_with_nutrition.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 320.0]</t>
+          <t>[35.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6077,7 @@
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6223,7 @@
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6296,7 @@
       </c>
       <c r="W80" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6661,7 @@
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="W87" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="W88" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="W90" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7099,7 +7099,7 @@
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7172,7 +7172,7 @@
       </c>
       <c r="W92" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7318,7 +7318,7 @@
       </c>
       <c r="W94" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7391,7 +7391,7 @@
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="W96" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7537,7 +7537,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7683,7 +7683,7 @@
       </c>
       <c r="W99" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="W100" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="W101" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8048,7 +8048,7 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="W105" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="W106" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8267,7 +8267,7 @@
       </c>
       <c r="W107" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="W108" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8413,7 +8413,7 @@
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8632,7 +8632,7 @@
       </c>
       <c r="W112" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="W113" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="W114" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="W115" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8924,7 +8924,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8997,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="W119" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9216,7 +9216,7 @@
       </c>
       <c r="W120" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="W121" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9362,7 +9362,7 @@
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
       </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -9508,7 +9508,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9581,7 +9581,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9654,7 +9654,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9800,7 +9800,7 @@
       </c>
       <c r="W128" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9873,7 +9873,7 @@
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="W130" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10019,7 +10019,7 @@
       </c>
       <c r="W131" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10165,7 +10165,7 @@
       </c>
       <c r="W133" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 320.0]</t>
+          <t>[35.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10238,7 @@
       </c>
       <c r="W134" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10311,7 +10311,7 @@
       </c>
       <c r="W135" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="W137" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10530,7 +10530,7 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="W139" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10749,7 @@
       </c>
       <c r="W141" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10895,7 +10895,7 @@
       </c>
       <c r="W143" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="W144" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11041,7 +11041,7 @@
       </c>
       <c r="W145" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="W146" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11187,7 +11187,7 @@
       </c>
       <c r="W147" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11260,7 @@
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11333,7 +11333,7 @@
       </c>
       <c r="W149" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11406,7 +11406,7 @@
       </c>
       <c r="W150" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11479,7 +11479,7 @@
       </c>
       <c r="W151" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="W152" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11625,7 +11625,7 @@
       </c>
       <c r="W153" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11698,7 @@
       </c>
       <c r="W154" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="W156" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="W157" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="W158" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="W159" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12136,7 +12136,7 @@
       </c>
       <c r="W160" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12209,7 +12209,7 @@
       </c>
       <c r="W161" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12282,7 +12282,7 @@
       </c>
       <c r="W162" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12355,7 +12355,7 @@
       </c>
       <c r="W163" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12428,7 +12428,7 @@
       </c>
       <c r="W164" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12501,7 +12501,7 @@
       </c>
       <c r="W165" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12574,7 +12574,7 @@
       </c>
       <c r="W166" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="W167" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12720,7 +12720,7 @@
       </c>
       <c r="W168" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12793,7 +12793,7 @@
       </c>
       <c r="W169" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12866,7 +12866,7 @@
       </c>
       <c r="W170" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -12939,7 +12939,7 @@
       </c>
       <c r="W171" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13012,7 +13012,7 @@
       </c>
       <c r="W172" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="W173" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13158,7 +13158,7 @@
       </c>
       <c r="W174" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="W175" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13304,7 +13304,7 @@
       </c>
       <c r="W176" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13377,7 +13377,7 @@
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13450,7 +13450,7 @@
       </c>
       <c r="W178" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13523,7 +13523,7 @@
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13596,7 +13596,7 @@
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13742,7 +13742,7 @@
       </c>
       <c r="W182" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13815,7 +13815,7 @@
       </c>
       <c r="W183" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13888,7 +13888,7 @@
       </c>
       <c r="W184" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -13961,7 +13961,7 @@
       </c>
       <c r="W185" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="W186" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14107,7 +14107,7 @@
       </c>
       <c r="W187" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14180,7 +14180,7 @@
       </c>
       <c r="W188" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14253,7 +14253,7 @@
       </c>
       <c r="W189" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14326,7 +14326,7 @@
       </c>
       <c r="W190" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14399,7 +14399,7 @@
       </c>
       <c r="W191" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14472,7 +14472,7 @@
       </c>
       <c r="W192" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14545,7 +14545,7 @@
       </c>
       <c r="W193" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14691,7 +14691,7 @@
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14764,7 +14764,7 @@
       </c>
       <c r="W196" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14837,7 +14837,7 @@
       </c>
       <c r="W197" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14910,7 +14910,7 @@
       </c>
       <c r="W198" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14983,7 +14983,7 @@
       </c>
       <c r="W199" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15056,7 +15056,7 @@
       </c>
       <c r="W200" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15129,7 +15129,7 @@
       </c>
       <c r="W201" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15202,7 +15202,7 @@
       </c>
       <c r="W202" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -15275,7 +15275,7 @@
       </c>
       <c r="W203" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -15348,7 +15348,7 @@
       </c>
       <c r="W204" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15421,7 +15421,7 @@
       </c>
       <c r="W205" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15494,7 +15494,7 @@
       </c>
       <c r="W206" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15567,7 +15567,7 @@
       </c>
       <c r="W207" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="W208" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -15713,7 +15713,7 @@
       </c>
       <c r="W209" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15786,7 +15786,7 @@
       </c>
       <c r="W210" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="W211" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15932,7 +15932,7 @@
       </c>
       <c r="W212" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="W213" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16078,7 +16078,7 @@
       </c>
       <c r="W214" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16151,7 +16151,7 @@
       </c>
       <c r="W215" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="W216" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16297,7 +16297,7 @@
       </c>
       <c r="W217" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16370,7 +16370,7 @@
       </c>
       <c r="W218" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16443,7 +16443,7 @@
       </c>
       <c r="W219" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16516,7 +16516,7 @@
       </c>
       <c r="W220" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16589,7 +16589,7 @@
       </c>
       <c r="W221" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16662,7 +16662,7 @@
       </c>
       <c r="W222" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16735,7 +16735,7 @@
       </c>
       <c r="W223" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16808,7 +16808,7 @@
       </c>
       <c r="W224" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16881,7 +16881,7 @@
       </c>
       <c r="W225" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16954,7 +16954,7 @@
       </c>
       <c r="W226" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17027,7 +17027,7 @@
       </c>
       <c r="W227" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17100,7 +17100,7 @@
       </c>
       <c r="W228" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17173,7 +17173,7 @@
       </c>
       <c r="W229" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17246,7 +17246,7 @@
       </c>
       <c r="W230" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17319,7 +17319,7 @@
       </c>
       <c r="W231" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17392,7 +17392,7 @@
       </c>
       <c r="W232" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17465,7 +17465,7 @@
       </c>
       <c r="W233" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17538,7 +17538,7 @@
       </c>
       <c r="W234" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17611,7 +17611,7 @@
       </c>
       <c r="W235" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17684,7 +17684,7 @@
       </c>
       <c r="W236" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17757,7 +17757,7 @@
       </c>
       <c r="W237" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17830,7 +17830,7 @@
       </c>
       <c r="W238" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="W239" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17976,7 +17976,7 @@
       </c>
       <c r="W240" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18049,7 +18049,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18122,7 +18122,7 @@
       </c>
       <c r="W242" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 320.0]</t>
+          <t>[35.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18195,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18268,7 +18268,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18341,7 +18341,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18487,7 +18487,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18560,7 +18560,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18706,7 +18706,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18779,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18852,7 +18852,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18925,7 +18925,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18998,7 +18998,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19071,7 +19071,7 @@
       </c>
       <c r="W255" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19144,7 +19144,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19217,7 +19217,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19290,7 +19290,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19363,7 +19363,7 @@
       </c>
       <c r="W259" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19436,7 +19436,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19509,7 +19509,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19582,7 +19582,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19655,7 +19655,7 @@
       </c>
       <c r="W263" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19728,7 +19728,7 @@
       </c>
       <c r="W264" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="W265" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -19874,7 +19874,7 @@
       </c>
       <c r="W266" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19947,7 +19947,7 @@
       </c>
       <c r="W267" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20020,7 +20020,7 @@
       </c>
       <c r="W268" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20093,7 +20093,7 @@
       </c>
       <c r="W269" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20166,7 +20166,7 @@
       </c>
       <c r="W270" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20239,7 +20239,7 @@
       </c>
       <c r="W271" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20312,7 +20312,7 @@
       </c>
       <c r="W272" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20385,7 +20385,7 @@
       </c>
       <c r="W273" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20458,7 +20458,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20531,7 +20531,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20604,7 +20604,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20677,7 +20677,7 @@
       </c>
       <c r="W277" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -20750,7 +20750,7 @@
       </c>
       <c r="W278" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20823,7 +20823,7 @@
       </c>
       <c r="W279" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20896,7 +20896,7 @@
       </c>
       <c r="W280" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20969,7 +20969,7 @@
       </c>
       <c r="W281" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21042,7 +21042,7 @@
       </c>
       <c r="W282" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21115,7 +21115,7 @@
       </c>
       <c r="W283" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21188,7 +21188,7 @@
       </c>
       <c r="W284" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21261,7 +21261,7 @@
       </c>
       <c r="W285" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21334,7 +21334,7 @@
       </c>
       <c r="W286" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="W287" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21480,7 +21480,7 @@
       </c>
       <c r="W288" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21553,7 +21553,7 @@
       </c>
       <c r="W289" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21626,7 +21626,7 @@
       </c>
       <c r="W290" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21699,7 +21699,7 @@
       </c>
       <c r="W291" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21772,7 +21772,7 @@
       </c>
       <c r="W292" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21845,7 +21845,7 @@
       </c>
       <c r="W293" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21918,7 +21918,7 @@
       </c>
       <c r="W294" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="W295" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22064,7 +22064,7 @@
       </c>
       <c r="W296" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22137,7 +22137,7 @@
       </c>
       <c r="W297" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22210,7 +22210,7 @@
       </c>
       <c r="W298" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22283,7 +22283,7 @@
       </c>
       <c r="W299" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22356,7 +22356,7 @@
       </c>
       <c r="W300" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22429,7 +22429,7 @@
       </c>
       <c r="W301" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22502,7 +22502,7 @@
       </c>
       <c r="W302" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22575,7 +22575,7 @@
       </c>
       <c r="W303" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22648,7 +22648,7 @@
       </c>
       <c r="W304" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22721,7 +22721,7 @@
       </c>
       <c r="W305" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22794,7 +22794,7 @@
       </c>
       <c r="W306" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 320.0]</t>
+          <t>[35.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22867,7 +22867,7 @@
       </c>
       <c r="W307" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22940,7 +22940,7 @@
       </c>
       <c r="W308" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23013,7 +23013,7 @@
       </c>
       <c r="W309" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="W310" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23159,7 +23159,7 @@
       </c>
       <c r="W311" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23232,7 +23232,7 @@
       </c>
       <c r="W312" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23305,7 +23305,7 @@
       </c>
       <c r="W313" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23378,7 +23378,7 @@
       </c>
       <c r="W314" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23451,7 +23451,7 @@
       </c>
       <c r="W315" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23524,7 +23524,7 @@
       </c>
       <c r="W316" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23597,7 +23597,7 @@
       </c>
       <c r="W317" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23670,7 +23670,7 @@
       </c>
       <c r="W318" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23743,7 +23743,7 @@
       </c>
       <c r="W319" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23816,7 +23816,7 @@
       </c>
       <c r="W320" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23889,7 +23889,7 @@
       </c>
       <c r="W321" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23962,7 +23962,7 @@
       </c>
       <c r="W322" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24035,7 +24035,7 @@
       </c>
       <c r="W323" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24108,7 +24108,7 @@
       </c>
       <c r="W324" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24181,7 +24181,7 @@
       </c>
       <c r="W325" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24254,7 +24254,7 @@
       </c>
       <c r="W326" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24327,7 +24327,7 @@
       </c>
       <c r="W327" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24400,7 +24400,7 @@
       </c>
       <c r="W328" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24473,7 +24473,7 @@
       </c>
       <c r="W329" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24546,7 +24546,7 @@
       </c>
       <c r="W330" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24619,7 +24619,7 @@
       </c>
       <c r="W331" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 320.0]</t>
+          <t>[35.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
       </c>
       <c r="W332" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24765,7 +24765,7 @@
       </c>
       <c r="W333" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24838,7 +24838,7 @@
       </c>
       <c r="W334" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24911,7 +24911,7 @@
       </c>
       <c r="W335" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -24984,7 +24984,7 @@
       </c>
       <c r="W336" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -25057,7 +25057,7 @@
       </c>
       <c r="W337" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25130,7 +25130,7 @@
       </c>
       <c r="W338" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="W339" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25276,7 +25276,7 @@
       </c>
       <c r="W340" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25349,7 +25349,7 @@
       </c>
       <c r="W341" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25422,7 +25422,7 @@
       </c>
       <c r="W342" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -25495,7 +25495,7 @@
       </c>
       <c r="W343" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25568,7 +25568,7 @@
       </c>
       <c r="W344" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25641,7 +25641,7 @@
       </c>
       <c r="W345" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25714,7 +25714,7 @@
       </c>
       <c r="W346" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25787,7 +25787,7 @@
       </c>
       <c r="W347" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25860,7 +25860,7 @@
       </c>
       <c r="W348" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25933,7 +25933,7 @@
       </c>
       <c r="W349" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26006,7 +26006,7 @@
       </c>
       <c r="W350" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26079,7 +26079,7 @@
       </c>
       <c r="W351" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26152,7 +26152,7 @@
       </c>
       <c r="W352" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26225,7 +26225,7 @@
       </c>
       <c r="W353" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26298,7 +26298,7 @@
       </c>
       <c r="W354" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26371,7 +26371,7 @@
       </c>
       <c r="W355" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26444,7 +26444,7 @@
       </c>
       <c r="W356" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26517,7 +26517,7 @@
       </c>
       <c r="W357" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26590,7 +26590,7 @@
       </c>
       <c r="W358" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26663,7 +26663,7 @@
       </c>
       <c r="W359" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26736,7 +26736,7 @@
       </c>
       <c r="W360" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26809,7 +26809,7 @@
       </c>
       <c r="W361" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26882,7 +26882,7 @@
       </c>
       <c r="W362" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26955,7 +26955,7 @@
       </c>
       <c r="W363" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27028,7 +27028,7 @@
       </c>
       <c r="W364" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27101,7 +27101,7 @@
       </c>
       <c r="W365" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27174,7 +27174,7 @@
       </c>
       <c r="W366" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27247,7 +27247,7 @@
       </c>
       <c r="W367" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27320,7 +27320,7 @@
       </c>
       <c r="W368" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27393,7 +27393,7 @@
       </c>
       <c r="W369" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27466,7 +27466,7 @@
       </c>
       <c r="W370" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27539,7 +27539,7 @@
       </c>
       <c r="W371" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27612,7 +27612,7 @@
       </c>
       <c r="W372" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27685,7 +27685,7 @@
       </c>
       <c r="W373" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27758,7 +27758,7 @@
       </c>
       <c r="W374" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27831,7 +27831,7 @@
       </c>
       <c r="W375" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -27904,7 +27904,7 @@
       </c>
       <c r="W376" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27977,7 +27977,7 @@
       </c>
       <c r="W377" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28050,7 +28050,7 @@
       </c>
       <c r="W378" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28123,7 +28123,7 @@
       </c>
       <c r="W379" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28196,7 +28196,7 @@
       </c>
       <c r="W380" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28269,7 +28269,7 @@
       </c>
       <c r="W381" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28342,7 +28342,7 @@
       </c>
       <c r="W382" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28415,7 +28415,7 @@
       </c>
       <c r="W383" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28488,7 +28488,7 @@
       </c>
       <c r="W384" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28561,7 +28561,7 @@
       </c>
       <c r="W385" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28634,7 +28634,7 @@
       </c>
       <c r="W386" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28707,7 +28707,7 @@
       </c>
       <c r="W387" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28780,7 +28780,7 @@
       </c>
       <c r="W388" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28853,7 +28853,7 @@
       </c>
       <c r="W389" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28926,7 +28926,7 @@
       </c>
       <c r="W390" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -28999,7 +28999,7 @@
       </c>
       <c r="W391" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29072,7 +29072,7 @@
       </c>
       <c r="W392" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29145,7 +29145,7 @@
       </c>
       <c r="W393" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29218,7 +29218,7 @@
       </c>
       <c r="W394" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29291,7 +29291,7 @@
       </c>
       <c r="W395" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29364,7 +29364,7 @@
       </c>
       <c r="W396" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29437,7 +29437,7 @@
       </c>
       <c r="W397" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29510,7 +29510,7 @@
       </c>
       <c r="W398" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29583,7 +29583,7 @@
       </c>
       <c r="W399" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29656,7 +29656,7 @@
       </c>
       <c r="W400" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29729,7 +29729,7 @@
       </c>
       <c r="W401" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29802,7 +29802,7 @@
       </c>
       <c r="W402" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29875,7 +29875,7 @@
       </c>
       <c r="W403" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -29948,7 +29948,7 @@
       </c>
       <c r="W404" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30021,7 +30021,7 @@
       </c>
       <c r="W405" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30094,7 +30094,7 @@
       </c>
       <c r="W406" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30167,7 +30167,7 @@
       </c>
       <c r="W407" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30240,7 +30240,7 @@
       </c>
       <c r="W408" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30313,7 +30313,7 @@
       </c>
       <c r="W409" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30386,7 +30386,7 @@
       </c>
       <c r="W410" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30459,7 +30459,7 @@
       </c>
       <c r="W411" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30532,7 +30532,7 @@
       </c>
       <c r="W412" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30605,7 +30605,7 @@
       </c>
       <c r="W413" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30678,7 +30678,7 @@
       </c>
       <c r="W414" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 400.0]</t>
+          <t>[25.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30751,7 +30751,7 @@
       </c>
       <c r="W415" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30824,7 +30824,7 @@
       </c>
       <c r="W416" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30897,7 +30897,7 @@
       </c>
       <c r="W417" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -30970,7 +30970,7 @@
       </c>
       <c r="W418" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31043,7 +31043,7 @@
       </c>
       <c r="W419" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31116,7 +31116,7 @@
       </c>
       <c r="W420" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31189,7 +31189,7 @@
       </c>
       <c r="W421" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31262,7 +31262,7 @@
       </c>
       <c r="W422" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31335,7 +31335,7 @@
       </c>
       <c r="W423" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31408,7 +31408,7 @@
       </c>
       <c r="W424" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31481,7 +31481,7 @@
       </c>
       <c r="W425" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31554,7 +31554,7 @@
       </c>
       <c r="W426" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31627,7 +31627,7 @@
       </c>
       <c r="W427" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31700,7 +31700,7 @@
       </c>
       <c r="W428" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31773,7 +31773,7 @@
       </c>
       <c r="W429" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31846,7 +31846,7 @@
       </c>
       <c r="W430" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31919,7 +31919,7 @@
       </c>
       <c r="W431" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31992,7 +31992,7 @@
       </c>
       <c r="W432" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32065,7 +32065,7 @@
       </c>
       <c r="W433" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32138,7 +32138,7 @@
       </c>
       <c r="W434" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32211,7 +32211,7 @@
       </c>
       <c r="W435" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32284,7 +32284,7 @@
       </c>
       <c r="W436" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32357,7 +32357,7 @@
       </c>
       <c r="W437" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32430,7 +32430,7 @@
       </c>
       <c r="W438" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32503,7 +32503,7 @@
       </c>
       <c r="W439" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32576,7 +32576,7 @@
       </c>
       <c r="W440" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32649,7 +32649,7 @@
       </c>
       <c r="W441" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32722,7 +32722,7 @@
       </c>
       <c r="W442" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32795,7 +32795,7 @@
       </c>
       <c r="W443" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32868,7 +32868,7 @@
       </c>
       <c r="W444" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32941,7 +32941,7 @@
       </c>
       <c r="W445" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33014,7 +33014,7 @@
       </c>
       <c r="W446" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33087,7 +33087,7 @@
       </c>
       <c r="W447" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33160,7 +33160,7 @@
       </c>
       <c r="W448" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33233,7 +33233,7 @@
       </c>
       <c r="W449" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33306,7 +33306,7 @@
       </c>
       <c r="W450" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33379,7 +33379,7 @@
       </c>
       <c r="W451" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33452,7 +33452,7 @@
       </c>
       <c r="W452" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33525,7 +33525,7 @@
       </c>
       <c r="W453" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33598,7 +33598,7 @@
       </c>
       <c r="W454" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33671,7 +33671,7 @@
       </c>
       <c r="W455" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33744,7 +33744,7 @@
       </c>
       <c r="W456" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 320.0]</t>
+          <t>[35.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33817,7 +33817,7 @@
       </c>
       <c r="W457" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -33890,7 +33890,7 @@
       </c>
       <c r="W458" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33963,7 +33963,7 @@
       </c>
       <c r="W459" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34036,7 +34036,7 @@
       </c>
       <c r="W460" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34109,7 +34109,7 @@
       </c>
       <c r="W461" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34182,7 +34182,7 @@
       </c>
       <c r="W462" t="inlineStr">
         <is>
-          <t>[25.0, 2.8, 400.0]</t>
+          <t>[25.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34255,7 +34255,7 @@
       </c>
       <c r="W463" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34328,7 +34328,7 @@
       </c>
       <c r="W464" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34401,7 +34401,7 @@
       </c>
       <c r="W465" t="inlineStr">
         <is>
-          <t>[35.0, 1.3, 400.0]</t>
+          <t>[35.0, 12.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34474,7 +34474,7 @@
       </c>
       <c r="W466" t="inlineStr">
         <is>
-          <t>[25.0, 1.3, 320.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -34547,7 +34547,7 @@
       </c>
       <c r="W467" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34620,7 +34620,7 @@
       </c>
       <c r="W468" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34693,7 +34693,7 @@
       </c>
       <c r="W469" t="inlineStr">
         <is>
-          <t>[35.0, 2.8, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
I made the nutrition vector logic more complex to create a tiered nutrition system based on the severity level of specific bio markers.
</commit_message>
<xml_diff>
--- a/pcos_data_with_nutrition.xlsx
+++ b/pcos_data_with_nutrition.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 22.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 22.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 320.0]</t>
+          <t>[27.5, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 22.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[37.5, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2281,7 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[40.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 18.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 18.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 22.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 24.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 12.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 22.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="W59" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="W60" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 22.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="W62" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 22.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 24.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 18.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6077,7 @@
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 24.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6223,7 @@
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6296,7 @@
       </c>
       <c r="W80" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[37.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6661,7 @@
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[40.0, 12.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="W87" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="W88" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="W90" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7099,7 +7099,7 @@
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7172,7 +7172,7 @@
       </c>
       <c r="W92" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 22.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7318,7 +7318,7 @@
       </c>
       <c r="W94" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7391,7 +7391,7 @@
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="W96" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[40.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7537,7 +7537,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -7683,7 +7683,7 @@
       </c>
       <c r="W99" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="W100" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="W101" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -8048,7 +8048,7 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 22.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="W105" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="W106" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8267,7 +8267,7 @@
       </c>
       <c r="W107" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="W108" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8413,7 +8413,7 @@
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8632,7 +8632,7 @@
       </c>
       <c r="W112" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="W113" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 18.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="W114" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="W115" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -8924,7 +8924,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8997,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="W119" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -9216,7 +9216,7 @@
       </c>
       <c r="W120" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="W121" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[37.5, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9362,7 +9362,7 @@
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
       </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -9508,7 +9508,7 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 12.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -9581,7 +9581,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -9654,7 +9654,7 @@
       </c>
       <c r="W126" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9800,7 +9800,7 @@
       </c>
       <c r="W128" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -9873,7 +9873,7 @@
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="W130" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -10019,7 +10019,7 @@
       </c>
       <c r="W131" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -10165,7 +10165,7 @@
       </c>
       <c r="W133" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 320.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10238,7 @@
       </c>
       <c r="W134" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10311,7 +10311,7 @@
       </c>
       <c r="W135" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="W137" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10530,7 +10530,7 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="W139" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10749,7 +10749,7 @@
       </c>
       <c r="W141" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10895,7 +10895,7 @@
       </c>
       <c r="W143" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="W144" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11041,7 +11041,7 @@
       </c>
       <c r="W145" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="W146" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11187,7 +11187,7 @@
       </c>
       <c r="W147" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11260,7 @@
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[30.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11333,7 +11333,7 @@
       </c>
       <c r="W149" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -11406,7 +11406,7 @@
       </c>
       <c r="W150" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11479,7 +11479,7 @@
       </c>
       <c r="W151" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="W152" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11625,7 +11625,7 @@
       </c>
       <c r="W153" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[40.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11698,7 @@
       </c>
       <c r="W154" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="W155" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11844,7 +11844,7 @@
       </c>
       <c r="W156" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="W157" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="W158" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 22.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="W159" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12136,7 +12136,7 @@
       </c>
       <c r="W160" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12209,7 +12209,7 @@
       </c>
       <c r="W161" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12282,7 +12282,7 @@
       </c>
       <c r="W162" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12428,7 +12428,7 @@
       </c>
       <c r="W164" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12501,7 +12501,7 @@
       </c>
       <c r="W165" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -12574,7 +12574,7 @@
       </c>
       <c r="W166" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="W167" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -12720,7 +12720,7 @@
       </c>
       <c r="W168" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12793,7 +12793,7 @@
       </c>
       <c r="W169" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12866,7 +12866,7 @@
       </c>
       <c r="W170" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -12939,7 +12939,7 @@
       </c>
       <c r="W171" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13012,7 +13012,7 @@
       </c>
       <c r="W172" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="W173" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -13158,7 +13158,7 @@
       </c>
       <c r="W174" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="W175" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -13304,7 +13304,7 @@
       </c>
       <c r="W176" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -13377,7 +13377,7 @@
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -13450,7 +13450,7 @@
       </c>
       <c r="W178" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -13523,7 +13523,7 @@
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -13596,7 +13596,7 @@
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13742,7 +13742,7 @@
       </c>
       <c r="W182" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13815,7 +13815,7 @@
       </c>
       <c r="W183" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -13888,7 +13888,7 @@
       </c>
       <c r="W184" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 22.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13961,7 +13961,7 @@
       </c>
       <c r="W185" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="W186" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 22.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -14107,7 +14107,7 @@
       </c>
       <c r="W187" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14180,7 +14180,7 @@
       </c>
       <c r="W188" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14253,7 +14253,7 @@
       </c>
       <c r="W189" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14326,7 +14326,7 @@
       </c>
       <c r="W190" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14399,7 +14399,7 @@
       </c>
       <c r="W191" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 22.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14472,7 +14472,7 @@
       </c>
       <c r="W192" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -14545,7 +14545,7 @@
       </c>
       <c r="W193" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -14691,7 +14691,7 @@
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -14764,7 +14764,7 @@
       </c>
       <c r="W196" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -14837,7 +14837,7 @@
       </c>
       <c r="W197" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -14910,7 +14910,7 @@
       </c>
       <c r="W198" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14983,7 +14983,7 @@
       </c>
       <c r="W199" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -15056,7 +15056,7 @@
       </c>
       <c r="W200" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15129,7 +15129,7 @@
       </c>
       <c r="W201" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15202,7 +15202,7 @@
       </c>
       <c r="W202" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 22.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -15275,7 +15275,7 @@
       </c>
       <c r="W203" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -15348,7 +15348,7 @@
       </c>
       <c r="W204" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15421,7 +15421,7 @@
       </c>
       <c r="W205" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -15494,7 +15494,7 @@
       </c>
       <c r="W206" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -15567,7 +15567,7 @@
       </c>
       <c r="W207" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="W208" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -15713,7 +15713,7 @@
       </c>
       <c r="W209" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 18.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -15786,7 +15786,7 @@
       </c>
       <c r="W210" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="W211" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -15932,7 +15932,7 @@
       </c>
       <c r="W212" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="W213" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -16078,7 +16078,7 @@
       </c>
       <c r="W214" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16151,7 +16151,7 @@
       </c>
       <c r="W215" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="W216" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 18.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -16297,7 +16297,7 @@
       </c>
       <c r="W217" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16370,7 +16370,7 @@
       </c>
       <c r="W218" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -16443,7 +16443,7 @@
       </c>
       <c r="W219" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -16516,7 +16516,7 @@
       </c>
       <c r="W220" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -16589,7 +16589,7 @@
       </c>
       <c r="W221" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16662,7 +16662,7 @@
       </c>
       <c r="W222" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -16735,7 +16735,7 @@
       </c>
       <c r="W223" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -16808,7 +16808,7 @@
       </c>
       <c r="W224" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 18.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16881,7 +16881,7 @@
       </c>
       <c r="W225" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 22.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -16954,7 +16954,7 @@
       </c>
       <c r="W226" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 18.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17100,7 +17100,7 @@
       </c>
       <c r="W228" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 22.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17173,7 +17173,7 @@
       </c>
       <c r="W229" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -17246,7 +17246,7 @@
       </c>
       <c r="W230" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -17319,7 +17319,7 @@
       </c>
       <c r="W231" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17465,7 +17465,7 @@
       </c>
       <c r="W233" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -17538,7 +17538,7 @@
       </c>
       <c r="W234" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17611,7 +17611,7 @@
       </c>
       <c r="W235" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -17684,7 +17684,7 @@
       </c>
       <c r="W236" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -17757,7 +17757,7 @@
       </c>
       <c r="W237" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17830,7 +17830,7 @@
       </c>
       <c r="W238" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="W239" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -17976,7 +17976,7 @@
       </c>
       <c r="W240" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18049,7 +18049,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -18122,7 +18122,7 @@
       </c>
       <c r="W242" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 320.0]</t>
+          <t>[32.5, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18195,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -18268,7 +18268,7 @@
       </c>
       <c r="W244" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -18341,7 +18341,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -18414,7 +18414,7 @@
       </c>
       <c r="W246" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18487,7 +18487,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -18560,7 +18560,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18706,7 +18706,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18779,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18852,7 +18852,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 22.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -18925,7 +18925,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -18998,7 +18998,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -19144,7 +19144,7 @@
       </c>
       <c r="W256" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -19217,7 +19217,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19290,7 +19290,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19436,7 +19436,7 @@
       </c>
       <c r="W260" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -19509,7 +19509,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -19582,7 +19582,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -19655,7 +19655,7 @@
       </c>
       <c r="W263" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 18.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -19728,7 +19728,7 @@
       </c>
       <c r="W264" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="W265" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -19874,7 +19874,7 @@
       </c>
       <c r="W266" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19947,7 +19947,7 @@
       </c>
       <c r="W267" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -20020,7 +20020,7 @@
       </c>
       <c r="W268" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -20093,7 +20093,7 @@
       </c>
       <c r="W269" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20166,7 +20166,7 @@
       </c>
       <c r="W270" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20239,7 +20239,7 @@
       </c>
       <c r="W271" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -20312,7 +20312,7 @@
       </c>
       <c r="W272" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -20385,7 +20385,7 @@
       </c>
       <c r="W273" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20458,7 +20458,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -20531,7 +20531,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -20604,7 +20604,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -20677,7 +20677,7 @@
       </c>
       <c r="W277" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -20750,7 +20750,7 @@
       </c>
       <c r="W278" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20823,7 +20823,7 @@
       </c>
       <c r="W279" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20896,7 +20896,7 @@
       </c>
       <c r="W280" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -20969,7 +20969,7 @@
       </c>
       <c r="W281" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21042,7 +21042,7 @@
       </c>
       <c r="W282" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -21115,7 +21115,7 @@
       </c>
       <c r="W283" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[37.5, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -21188,7 +21188,7 @@
       </c>
       <c r="W284" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -21261,7 +21261,7 @@
       </c>
       <c r="W285" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -21334,7 +21334,7 @@
       </c>
       <c r="W286" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="W287" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -21480,7 +21480,7 @@
       </c>
       <c r="W288" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -21553,7 +21553,7 @@
       </c>
       <c r="W289" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21626,7 +21626,7 @@
       </c>
       <c r="W290" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 22.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21699,7 +21699,7 @@
       </c>
       <c r="W291" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 24.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21772,7 +21772,7 @@
       </c>
       <c r="W292" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -21845,7 +21845,7 @@
       </c>
       <c r="W293" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -21918,7 +21918,7 @@
       </c>
       <c r="W294" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="W295" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -22064,7 +22064,7 @@
       </c>
       <c r="W296" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22210,7 +22210,7 @@
       </c>
       <c r="W298" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -22283,7 +22283,7 @@
       </c>
       <c r="W299" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -22356,7 +22356,7 @@
       </c>
       <c r="W300" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22429,7 +22429,7 @@
       </c>
       <c r="W301" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -22502,7 +22502,7 @@
       </c>
       <c r="W302" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -22575,7 +22575,7 @@
       </c>
       <c r="W303" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22648,7 +22648,7 @@
       </c>
       <c r="W304" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -22721,7 +22721,7 @@
       </c>
       <c r="W305" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22794,7 +22794,7 @@
       </c>
       <c r="W306" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 320.0]</t>
+          <t>[32.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -22867,7 +22867,7 @@
       </c>
       <c r="W307" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22940,7 +22940,7 @@
       </c>
       <c r="W308" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -23013,7 +23013,7 @@
       </c>
       <c r="W309" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 22.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="W310" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -23159,7 +23159,7 @@
       </c>
       <c r="W311" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23232,7 +23232,7 @@
       </c>
       <c r="W312" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -23305,7 +23305,7 @@
       </c>
       <c r="W313" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23378,7 +23378,7 @@
       </c>
       <c r="W314" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -23451,7 +23451,7 @@
       </c>
       <c r="W315" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 22.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23524,7 +23524,7 @@
       </c>
       <c r="W316" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -23597,7 +23597,7 @@
       </c>
       <c r="W317" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 22.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23670,7 +23670,7 @@
       </c>
       <c r="W318" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23743,7 +23743,7 @@
       </c>
       <c r="W319" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 24.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23816,7 +23816,7 @@
       </c>
       <c r="W320" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 22.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -23889,7 +23889,7 @@
       </c>
       <c r="W321" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23962,7 +23962,7 @@
       </c>
       <c r="W322" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24108,7 +24108,7 @@
       </c>
       <c r="W324" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -24181,7 +24181,7 @@
       </c>
       <c r="W325" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -24254,7 +24254,7 @@
       </c>
       <c r="W326" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -24327,7 +24327,7 @@
       </c>
       <c r="W327" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24400,7 +24400,7 @@
       </c>
       <c r="W328" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -24473,7 +24473,7 @@
       </c>
       <c r="W329" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -24546,7 +24546,7 @@
       </c>
       <c r="W330" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 18.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -24619,7 +24619,7 @@
       </c>
       <c r="W331" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 320.0]</t>
+          <t>[27.5, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
       </c>
       <c r="W332" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -24765,7 +24765,7 @@
       </c>
       <c r="W333" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -24838,7 +24838,7 @@
       </c>
       <c r="W334" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -24911,7 +24911,7 @@
       </c>
       <c r="W335" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -24984,7 +24984,7 @@
       </c>
       <c r="W336" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[35.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -25057,7 +25057,7 @@
       </c>
       <c r="W337" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -25130,7 +25130,7 @@
       </c>
       <c r="W338" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="W339" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25276,7 +25276,7 @@
       </c>
       <c r="W340" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -25349,7 +25349,7 @@
       </c>
       <c r="W341" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -25495,7 +25495,7 @@
       </c>
       <c r="W343" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -25568,7 +25568,7 @@
       </c>
       <c r="W344" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25641,7 +25641,7 @@
       </c>
       <c r="W345" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 24.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25714,7 +25714,7 @@
       </c>
       <c r="W346" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -25787,7 +25787,7 @@
       </c>
       <c r="W347" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25860,7 +25860,7 @@
       </c>
       <c r="W348" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25933,7 +25933,7 @@
       </c>
       <c r="W349" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -26006,7 +26006,7 @@
       </c>
       <c r="W350" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -26079,7 +26079,7 @@
       </c>
       <c r="W351" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26152,7 +26152,7 @@
       </c>
       <c r="W352" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -26225,7 +26225,7 @@
       </c>
       <c r="W353" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -26298,7 +26298,7 @@
       </c>
       <c r="W354" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -26371,7 +26371,7 @@
       </c>
       <c r="W355" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26444,7 +26444,7 @@
       </c>
       <c r="W356" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 18.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26517,7 +26517,7 @@
       </c>
       <c r="W357" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -26590,7 +26590,7 @@
       </c>
       <c r="W358" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -26663,7 +26663,7 @@
       </c>
       <c r="W359" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -26736,7 +26736,7 @@
       </c>
       <c r="W360" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26809,7 +26809,7 @@
       </c>
       <c r="W361" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 22.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26882,7 +26882,7 @@
       </c>
       <c r="W362" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26955,7 +26955,7 @@
       </c>
       <c r="W363" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27028,7 +27028,7 @@
       </c>
       <c r="W364" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27101,7 +27101,7 @@
       </c>
       <c r="W365" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27174,7 +27174,7 @@
       </c>
       <c r="W366" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27247,7 +27247,7 @@
       </c>
       <c r="W367" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27320,7 +27320,7 @@
       </c>
       <c r="W368" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27393,7 +27393,7 @@
       </c>
       <c r="W369" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27466,7 +27466,7 @@
       </c>
       <c r="W370" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27539,7 +27539,7 @@
       </c>
       <c r="W371" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -27612,7 +27612,7 @@
       </c>
       <c r="W372" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 18.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -27685,7 +27685,7 @@
       </c>
       <c r="W373" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 24.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27758,7 +27758,7 @@
       </c>
       <c r="W374" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -27831,7 +27831,7 @@
       </c>
       <c r="W375" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -27904,7 +27904,7 @@
       </c>
       <c r="W376" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[35.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27977,7 +27977,7 @@
       </c>
       <c r="W377" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -28050,7 +28050,7 @@
       </c>
       <c r="W378" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -28123,7 +28123,7 @@
       </c>
       <c r="W379" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -28196,7 +28196,7 @@
       </c>
       <c r="W380" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28269,7 +28269,7 @@
       </c>
       <c r="W381" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -28342,7 +28342,7 @@
       </c>
       <c r="W382" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -28415,7 +28415,7 @@
       </c>
       <c r="W383" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -28488,7 +28488,7 @@
       </c>
       <c r="W384" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -28561,7 +28561,7 @@
       </c>
       <c r="W385" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28634,7 +28634,7 @@
       </c>
       <c r="W386" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28707,7 +28707,7 @@
       </c>
       <c r="W387" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -28780,7 +28780,7 @@
       </c>
       <c r="W388" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -28853,7 +28853,7 @@
       </c>
       <c r="W389" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -28926,7 +28926,7 @@
       </c>
       <c r="W390" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -28999,7 +28999,7 @@
       </c>
       <c r="W391" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29072,7 +29072,7 @@
       </c>
       <c r="W392" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29145,7 +29145,7 @@
       </c>
       <c r="W393" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29218,7 +29218,7 @@
       </c>
       <c r="W394" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -29291,7 +29291,7 @@
       </c>
       <c r="W395" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -29364,7 +29364,7 @@
       </c>
       <c r="W396" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29437,7 +29437,7 @@
       </c>
       <c r="W397" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -29510,7 +29510,7 @@
       </c>
       <c r="W398" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29583,7 +29583,7 @@
       </c>
       <c r="W399" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29656,7 +29656,7 @@
       </c>
       <c r="W400" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -29729,7 +29729,7 @@
       </c>
       <c r="W401" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29802,7 +29802,7 @@
       </c>
       <c r="W402" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 24.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29875,7 +29875,7 @@
       </c>
       <c r="W403" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29948,7 +29948,7 @@
       </c>
       <c r="W404" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30021,7 +30021,7 @@
       </c>
       <c r="W405" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30094,7 +30094,7 @@
       </c>
       <c r="W406" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30167,7 +30167,7 @@
       </c>
       <c r="W407" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30240,7 +30240,7 @@
       </c>
       <c r="W408" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30313,7 +30313,7 @@
       </c>
       <c r="W409" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30386,7 +30386,7 @@
       </c>
       <c r="W410" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30459,7 +30459,7 @@
       </c>
       <c r="W411" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30532,7 +30532,7 @@
       </c>
       <c r="W412" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30605,7 +30605,7 @@
       </c>
       <c r="W413" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30678,7 +30678,7 @@
       </c>
       <c r="W414" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30824,7 +30824,7 @@
       </c>
       <c r="W416" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -30897,7 +30897,7 @@
       </c>
       <c r="W417" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 24.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30970,7 +30970,7 @@
       </c>
       <c r="W418" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31043,7 +31043,7 @@
       </c>
       <c r="W419" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -31189,7 +31189,7 @@
       </c>
       <c r="W421" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[25.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31262,7 +31262,7 @@
       </c>
       <c r="W422" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 18.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -31335,7 +31335,7 @@
       </c>
       <c r="W423" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -31408,7 +31408,7 @@
       </c>
       <c r="W424" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -31554,7 +31554,7 @@
       </c>
       <c r="W426" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -31627,7 +31627,7 @@
       </c>
       <c r="W427" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -31700,7 +31700,7 @@
       </c>
       <c r="W428" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31773,7 +31773,7 @@
       </c>
       <c r="W429" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[27.5, 24.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31846,7 +31846,7 @@
       </c>
       <c r="W430" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -31919,7 +31919,7 @@
       </c>
       <c r="W431" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31992,7 +31992,7 @@
       </c>
       <c r="W432" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32065,7 +32065,7 @@
       </c>
       <c r="W433" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -32138,7 +32138,7 @@
       </c>
       <c r="W434" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 22.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -32211,7 +32211,7 @@
       </c>
       <c r="W435" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 22.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32284,7 +32284,7 @@
       </c>
       <c r="W436" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -32357,7 +32357,7 @@
       </c>
       <c r="W437" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 22.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32430,7 +32430,7 @@
       </c>
       <c r="W438" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -32503,7 +32503,7 @@
       </c>
       <c r="W439" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 18.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32576,7 +32576,7 @@
       </c>
       <c r="W440" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -32649,7 +32649,7 @@
       </c>
       <c r="W441" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[37.5, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -32722,7 +32722,7 @@
       </c>
       <c r="W442" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 18.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -32795,7 +32795,7 @@
       </c>
       <c r="W443" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -32868,7 +32868,7 @@
       </c>
       <c r="W444" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32941,7 +32941,7 @@
       </c>
       <c r="W445" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -33014,7 +33014,7 @@
       </c>
       <c r="W446" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33087,7 +33087,7 @@
       </c>
       <c r="W447" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33160,7 +33160,7 @@
       </c>
       <c r="W448" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -33233,7 +33233,7 @@
       </c>
       <c r="W449" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33306,7 +33306,7 @@
       </c>
       <c r="W450" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 22.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33379,7 +33379,7 @@
       </c>
       <c r="W451" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33452,7 +33452,7 @@
       </c>
       <c r="W452" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33525,7 +33525,7 @@
       </c>
       <c r="W453" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33598,7 +33598,7 @@
       </c>
       <c r="W454" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[27.5, 22.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33671,7 +33671,7 @@
       </c>
       <c r="W455" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33744,7 +33744,7 @@
       </c>
       <c r="W456" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 320.0]</t>
+          <t>[37.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -33817,7 +33817,7 @@
       </c>
       <c r="W457" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33890,7 +33890,7 @@
       </c>
       <c r="W458" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 18.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33963,7 +33963,7 @@
       </c>
       <c r="W459" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[35.0, 18.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34036,7 +34036,7 @@
       </c>
       <c r="W460" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[30.0, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -34109,7 +34109,7 @@
       </c>
       <c r="W461" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -34182,7 +34182,7 @@
       </c>
       <c r="W462" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 400.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -34255,7 +34255,7 @@
       </c>
       <c r="W463" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[25.0, 24.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -34401,7 +34401,7 @@
       </c>
       <c r="W465" t="inlineStr">
         <is>
-          <t>[35.0, 12.0, 400.0]</t>
+          <t>[37.5, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34474,7 +34474,7 @@
       </c>
       <c r="W466" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[25.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -34547,7 +34547,7 @@
       </c>
       <c r="W467" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 22.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -34620,7 +34620,7 @@
       </c>
       <c r="W468" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[40.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -34693,7 +34693,7 @@
       </c>
       <c r="W469" t="inlineStr">
         <is>
-          <t>[35.0, 20.0, 400.0]</t>
+          <t>[30.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed the nutrition vector logic with if and elif statements
</commit_message>
<xml_diff>
--- a/pcos_data_with_nutrition.xlsx
+++ b/pcos_data_with_nutrition.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>[40.0, 20.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 355.0]</t>
+          <t>[30.0, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>[32.5, 22.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 320.0]</t>
+          <t>[30.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>[37.5, 22.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>[40.0, 14.0, 360.0]</t>
+          <t>[35.0, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2719,7 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 320.0]</t>
+          <t>[32.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 360.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>[40.0, 20.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>[40.0, 18.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 355.0]</t>
+          <t>[30.0, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 320.0]</t>
+          <t>[32.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>[40.0, 24.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="W53" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 360.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4544,7 @@
       </c>
       <c r="W56" t="inlineStr">
         <is>
-          <t>[32.5, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>[35.0, 22.0, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="W61" t="inlineStr">
         <is>
-          <t>[32.5, 22.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="W63" t="inlineStr">
         <is>
-          <t>[40.0, 16.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="W64" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>[32.5, 22.0, 355.0]</t>
+          <t>[32.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="W69" t="inlineStr">
         <is>
-          <t>[27.5, 24.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5566,7 @@
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>[37.5, 20.0, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>[40.0, 18.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>[40.0, 16.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="W76" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>[27.5, 24.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6223,7 @@
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="W81" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="W82" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 360.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -6515,7 +6515,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 355.0]</t>
+          <t>[35.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6661,7 @@
       </c>
       <c r="W85" t="inlineStr">
         <is>
-          <t>[40.0, 12.0, 390.0]</t>
+          <t>[35.0, 12.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -6807,7 +6807,7 @@
       </c>
       <c r="W87" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="W88" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="W90" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7172,7 +7172,7 @@
       </c>
       <c r="W92" t="inlineStr">
         <is>
-          <t>[25.0, 22.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7391,7 +7391,7 @@
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="W96" t="inlineStr">
         <is>
-          <t>[40.0, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -7537,7 +7537,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="W100" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="W101" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -7975,7 +7975,7 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -8048,7 +8048,7 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>[25.0, 22.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8413,7 +8413,7 @@
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8486,7 @@
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="W113" t="inlineStr">
         <is>
-          <t>[40.0, 18.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="W114" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="W115" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -8924,7 +8924,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9143,7 @@
       </c>
       <c r="W119" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -9216,7 +9216,7 @@
       </c>
       <c r="W120" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="W121" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9581,7 +9581,7 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="W127" t="inlineStr">
         <is>
-          <t>[40.0, 16.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -9800,7 +9800,7 @@
       </c>
       <c r="W128" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -9873,7 +9873,7 @@
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="W130" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -10165,7 +10165,7 @@
       </c>
       <c r="W133" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10238,7 @@
       </c>
       <c r="W134" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="W137" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -10530,7 +10530,7 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10603,7 @@
       </c>
       <c r="W139" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -10822,7 +10822,7 @@
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 345.0]</t>
+          <t>[30.0, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="W144" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -11041,7 +11041,7 @@
       </c>
       <c r="W145" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11187,7 +11187,7 @@
       </c>
       <c r="W147" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11260,7 @@
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 320.0]</t>
+          <t>[32.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11333,7 +11333,7 @@
       </c>
       <c r="W149" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -11406,7 +11406,7 @@
       </c>
       <c r="W150" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11479,7 +11479,7 @@
       </c>
       <c r="W151" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 320.0]</t>
+          <t>[30.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="W152" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -11625,7 +11625,7 @@
       </c>
       <c r="W153" t="inlineStr">
         <is>
-          <t>[40.0, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="W157" t="inlineStr">
         <is>
-          <t>[40.0, 20.0, 370.0]</t>
+          <t>[35.0, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -11990,7 +11990,7 @@
       </c>
       <c r="W158" t="inlineStr">
         <is>
-          <t>[32.5, 22.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12136,7 +12136,7 @@
       </c>
       <c r="W160" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12209,7 +12209,7 @@
       </c>
       <c r="W161" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 320.0]</t>
+          <t>[32.5, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12282,7 +12282,7 @@
       </c>
       <c r="W162" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12428,7 +12428,7 @@
       </c>
       <c r="W164" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12501,7 +12501,7 @@
       </c>
       <c r="W165" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -12647,7 +12647,7 @@
       </c>
       <c r="W167" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -12720,7 +12720,7 @@
       </c>
       <c r="W168" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -12793,7 +12793,7 @@
       </c>
       <c r="W169" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 320.0]</t>
+          <t>[30.0, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -12866,7 +12866,7 @@
       </c>
       <c r="W170" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -12939,7 +12939,7 @@
       </c>
       <c r="W171" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="W173" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -13158,7 +13158,7 @@
       </c>
       <c r="W174" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="W175" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -13304,7 +13304,7 @@
       </c>
       <c r="W176" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -13377,7 +13377,7 @@
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -13450,7 +13450,7 @@
       </c>
       <c r="W178" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -13523,7 +13523,7 @@
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -13596,7 +13596,7 @@
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13742,7 +13742,7 @@
       </c>
       <c r="W182" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13888,7 +13888,7 @@
       </c>
       <c r="W184" t="inlineStr">
         <is>
-          <t>[32.5, 22.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -13961,7 +13961,7 @@
       </c>
       <c r="W185" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="W186" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -14107,7 +14107,7 @@
       </c>
       <c r="W187" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14399,7 +14399,7 @@
       </c>
       <c r="W191" t="inlineStr">
         <is>
-          <t>[32.5, 22.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -14472,7 +14472,7 @@
       </c>
       <c r="W192" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -14618,7 +14618,7 @@
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -14691,7 +14691,7 @@
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -14837,7 +14837,7 @@
       </c>
       <c r="W197" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -14910,7 +14910,7 @@
       </c>
       <c r="W198" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -14983,7 +14983,7 @@
       </c>
       <c r="W199" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -15056,7 +15056,7 @@
       </c>
       <c r="W200" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15129,7 +15129,7 @@
       </c>
       <c r="W201" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -15202,7 +15202,7 @@
       </c>
       <c r="W202" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -15348,7 +15348,7 @@
       </c>
       <c r="W204" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15421,7 +15421,7 @@
       </c>
       <c r="W205" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -15567,7 +15567,7 @@
       </c>
       <c r="W207" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 360.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="W208" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -15713,7 +15713,7 @@
       </c>
       <c r="W209" t="inlineStr">
         <is>
-          <t>[32.5, 18.0, 355.0]</t>
+          <t>[32.5, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -15786,7 +15786,7 @@
       </c>
       <c r="W210" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 360.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="W211" t="inlineStr">
         <is>
-          <t>[37.5, 20.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="W213" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -16151,7 +16151,7 @@
       </c>
       <c r="W215" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="W216" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -16297,7 +16297,7 @@
       </c>
       <c r="W217" t="inlineStr">
         <is>
-          <t>[25.0, 14.0, 320.0]</t>
+          <t>[27.5, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -16516,7 +16516,7 @@
       </c>
       <c r="W220" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -16808,7 +16808,7 @@
       </c>
       <c r="W224" t="inlineStr">
         <is>
-          <t>[40.0, 18.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -16881,7 +16881,7 @@
       </c>
       <c r="W225" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -16954,7 +16954,7 @@
       </c>
       <c r="W226" t="inlineStr">
         <is>
-          <t>[37.5, 18.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -17100,7 +17100,7 @@
       </c>
       <c r="W228" t="inlineStr">
         <is>
-          <t>[25.0, 22.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -17173,7 +17173,7 @@
       </c>
       <c r="W229" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -17246,7 +17246,7 @@
       </c>
       <c r="W230" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -17465,7 +17465,7 @@
       </c>
       <c r="W233" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -17830,7 +17830,7 @@
       </c>
       <c r="W238" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -17903,7 +17903,7 @@
       </c>
       <c r="W239" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -17976,7 +17976,7 @@
       </c>
       <c r="W240" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18049,7 +18049,7 @@
       </c>
       <c r="W241" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18195,7 @@
       </c>
       <c r="W243" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -18341,7 +18341,7 @@
       </c>
       <c r="W245" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -18487,7 +18487,7 @@
       </c>
       <c r="W247" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -18560,7 +18560,7 @@
       </c>
       <c r="W248" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="W249" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -18706,7 +18706,7 @@
       </c>
       <c r="W250" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -18779,7 +18779,7 @@
       </c>
       <c r="W251" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -18852,7 +18852,7 @@
       </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>[30.0, 22.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -18925,7 +18925,7 @@
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -18998,7 +18998,7 @@
       </c>
       <c r="W254" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -19217,7 +19217,7 @@
       </c>
       <c r="W257" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 320.0]</t>
+          <t>[32.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19290,7 +19290,7 @@
       </c>
       <c r="W258" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 320.0]</t>
+          <t>[32.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -19509,7 +19509,7 @@
       </c>
       <c r="W261" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -19582,7 +19582,7 @@
       </c>
       <c r="W262" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 345.0]</t>
+          <t>[30.0, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -19655,7 +19655,7 @@
       </c>
       <c r="W263" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -19728,7 +19728,7 @@
       </c>
       <c r="W264" t="inlineStr">
         <is>
-          <t>[32.5, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="W265" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -19947,7 +19947,7 @@
       </c>
       <c r="W267" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -20020,7 +20020,7 @@
       </c>
       <c r="W268" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 345.0]</t>
+          <t>[30.0, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -20093,7 +20093,7 @@
       </c>
       <c r="W269" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20166,7 +20166,7 @@
       </c>
       <c r="W270" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20239,7 +20239,7 @@
       </c>
       <c r="W271" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -20385,7 +20385,7 @@
       </c>
       <c r="W273" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -20458,7 +20458,7 @@
       </c>
       <c r="W274" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -20531,7 +20531,7 @@
       </c>
       <c r="W275" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -20604,7 +20604,7 @@
       </c>
       <c r="W276" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -20750,7 +20750,7 @@
       </c>
       <c r="W278" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -20823,7 +20823,7 @@
       </c>
       <c r="W279" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -21042,7 +21042,7 @@
       </c>
       <c r="W282" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -21115,7 +21115,7 @@
       </c>
       <c r="W283" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -21188,7 +21188,7 @@
       </c>
       <c r="W284" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -21261,7 +21261,7 @@
       </c>
       <c r="W285" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -21334,7 +21334,7 @@
       </c>
       <c r="W286" t="inlineStr">
         <is>
-          <t>[40.0, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -21407,7 +21407,7 @@
       </c>
       <c r="W287" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -21480,7 +21480,7 @@
       </c>
       <c r="W288" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -21553,7 +21553,7 @@
       </c>
       <c r="W289" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 320.0]</t>
+          <t>[32.5, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21626,7 +21626,7 @@
       </c>
       <c r="W290" t="inlineStr">
         <is>
-          <t>[35.0, 22.0, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -21699,7 +21699,7 @@
       </c>
       <c r="W291" t="inlineStr">
         <is>
-          <t>[25.0, 24.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -21772,7 +21772,7 @@
       </c>
       <c r="W292" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -21845,7 +21845,7 @@
       </c>
       <c r="W293" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -21918,7 +21918,7 @@
       </c>
       <c r="W294" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="W295" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 390.0]</t>
+          <t>[35.0, 14.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -22064,7 +22064,7 @@
       </c>
       <c r="W296" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -22210,7 +22210,7 @@
       </c>
       <c r="W298" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -22283,7 +22283,7 @@
       </c>
       <c r="W299" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -22502,7 +22502,7 @@
       </c>
       <c r="W302" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -22648,7 +22648,7 @@
       </c>
       <c r="W304" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -22867,7 +22867,7 @@
       </c>
       <c r="W307" t="inlineStr">
         <is>
-          <t>[25.0, 16.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -22940,7 +22940,7 @@
       </c>
       <c r="W308" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 355.0]</t>
+          <t>[30.0, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -23013,7 +23013,7 @@
       </c>
       <c r="W309" t="inlineStr">
         <is>
-          <t>[30.0, 22.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="W310" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -23159,7 +23159,7 @@
       </c>
       <c r="W311" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23232,7 +23232,7 @@
       </c>
       <c r="W312" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -23378,7 +23378,7 @@
       </c>
       <c r="W314" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -23451,7 +23451,7 @@
       </c>
       <c r="W315" t="inlineStr">
         <is>
-          <t>[30.0, 22.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -23597,7 +23597,7 @@
       </c>
       <c r="W317" t="inlineStr">
         <is>
-          <t>[25.0, 22.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23743,7 +23743,7 @@
       </c>
       <c r="W319" t="inlineStr">
         <is>
-          <t>[25.0, 24.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23816,7 +23816,7 @@
       </c>
       <c r="W320" t="inlineStr">
         <is>
-          <t>[37.5, 22.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -23889,7 +23889,7 @@
       </c>
       <c r="W321" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -23962,7 +23962,7 @@
       </c>
       <c r="W322" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24181,7 +24181,7 @@
       </c>
       <c r="W325" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -24327,7 +24327,7 @@
       </c>
       <c r="W327" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 320.0]</t>
+          <t>[32.5, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24400,7 +24400,7 @@
       </c>
       <c r="W328" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -24473,7 +24473,7 @@
       </c>
       <c r="W329" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -24546,7 +24546,7 @@
       </c>
       <c r="W330" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -24619,7 +24619,7 @@
       </c>
       <c r="W331" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 320.0]</t>
+          <t>[30.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
       </c>
       <c r="W332" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 355.0]</t>
+          <t>[30.0, 12.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -24765,7 +24765,7 @@
       </c>
       <c r="W333" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -24838,7 +24838,7 @@
       </c>
       <c r="W334" t="inlineStr">
         <is>
-          <t>[27.5, 12.0, 345.0]</t>
+          <t>[30.0, 12.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -25057,7 +25057,7 @@
       </c>
       <c r="W337" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -25130,7 +25130,7 @@
       </c>
       <c r="W338" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25203,7 +25203,7 @@
       </c>
       <c r="W339" t="inlineStr">
         <is>
-          <t>[32.5, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25276,7 +25276,7 @@
       </c>
       <c r="W340" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -25349,7 +25349,7 @@
       </c>
       <c r="W341" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -25641,7 +25641,7 @@
       </c>
       <c r="W345" t="inlineStr">
         <is>
-          <t>[35.0, 24.0, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -25714,7 +25714,7 @@
       </c>
       <c r="W346" t="inlineStr">
         <is>
-          <t>[37.5, 20.0, 390.0]</t>
+          <t>[35.0, 20.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -25787,7 +25787,7 @@
       </c>
       <c r="W347" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25860,7 +25860,7 @@
       </c>
       <c r="W348" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -25933,7 +25933,7 @@
       </c>
       <c r="W349" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -26152,7 +26152,7 @@
       </c>
       <c r="W352" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -26225,7 +26225,7 @@
       </c>
       <c r="W353" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -26298,7 +26298,7 @@
       </c>
       <c r="W354" t="inlineStr">
         <is>
-          <t>[40.0, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -26444,7 +26444,7 @@
       </c>
       <c r="W356" t="inlineStr">
         <is>
-          <t>[37.5, 18.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -26517,7 +26517,7 @@
       </c>
       <c r="W357" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 355.0]</t>
+          <t>[30.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -26590,7 +26590,7 @@
       </c>
       <c r="W358" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -26663,7 +26663,7 @@
       </c>
       <c r="W359" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -26809,7 +26809,7 @@
       </c>
       <c r="W361" t="inlineStr">
         <is>
-          <t>[25.0, 22.0, 320.0]</t>
+          <t>[27.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -26955,7 +26955,7 @@
       </c>
       <c r="W363" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27101,7 +27101,7 @@
       </c>
       <c r="W365" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27174,7 +27174,7 @@
       </c>
       <c r="W366" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 320.0]</t>
+          <t>[30.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27320,7 +27320,7 @@
       </c>
       <c r="W368" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27393,7 +27393,7 @@
       </c>
       <c r="W369" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -27539,7 +27539,7 @@
       </c>
       <c r="W371" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -27612,7 +27612,7 @@
       </c>
       <c r="W372" t="inlineStr">
         <is>
-          <t>[35.0, 18.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -27685,7 +27685,7 @@
       </c>
       <c r="W373" t="inlineStr">
         <is>
-          <t>[30.0, 24.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -27758,7 +27758,7 @@
       </c>
       <c r="W374" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -27831,7 +27831,7 @@
       </c>
       <c r="W375" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -28050,7 +28050,7 @@
       </c>
       <c r="W378" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -28123,7 +28123,7 @@
       </c>
       <c r="W379" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -28196,7 +28196,7 @@
       </c>
       <c r="W380" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 320.0]</t>
+          <t>[32.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28342,7 +28342,7 @@
       </c>
       <c r="W382" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -28488,7 +28488,7 @@
       </c>
       <c r="W384" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -28561,7 +28561,7 @@
       </c>
       <c r="W385" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28634,7 +28634,7 @@
       </c>
       <c r="W386" t="inlineStr">
         <is>
-          <t>[25.0, 16.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -28707,7 +28707,7 @@
       </c>
       <c r="W387" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -28780,7 +28780,7 @@
       </c>
       <c r="W388" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -29072,7 +29072,7 @@
       </c>
       <c r="W392" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29145,7 +29145,7 @@
       </c>
       <c r="W393" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29218,7 +29218,7 @@
       </c>
       <c r="W394" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -29291,7 +29291,7 @@
       </c>
       <c r="W395" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -29364,7 +29364,7 @@
       </c>
       <c r="W396" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29437,7 +29437,7 @@
       </c>
       <c r="W397" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -29510,7 +29510,7 @@
       </c>
       <c r="W398" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 360.0]</t>
+          <t>[32.5, 12.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -29802,7 +29802,7 @@
       </c>
       <c r="W402" t="inlineStr">
         <is>
-          <t>[25.0, 24.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -29948,7 +29948,7 @@
       </c>
       <c r="W404" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30021,7 +30021,7 @@
       </c>
       <c r="W405" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 355.0]</t>
+          <t>[30.0, 16.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30167,7 +30167,7 @@
       </c>
       <c r="W407" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30240,7 +30240,7 @@
       </c>
       <c r="W408" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 360.0]</t>
+          <t>[32.5, 20.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30313,7 +30313,7 @@
       </c>
       <c r="W409" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30386,7 +30386,7 @@
       </c>
       <c r="W410" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -30532,7 +30532,7 @@
       </c>
       <c r="W412" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -30605,7 +30605,7 @@
       </c>
       <c r="W413" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30824,7 +30824,7 @@
       </c>
       <c r="W416" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -30897,7 +30897,7 @@
       </c>
       <c r="W417" t="inlineStr">
         <is>
-          <t>[32.5, 24.0, 355.0]</t>
+          <t>[32.5, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -30970,7 +30970,7 @@
       </c>
       <c r="W418" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31043,7 +31043,7 @@
       </c>
       <c r="W419" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -31189,7 +31189,7 @@
       </c>
       <c r="W421" t="inlineStr">
         <is>
-          <t>[25.0, 12.0, 320.0]</t>
+          <t>[27.5, 12.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31262,7 +31262,7 @@
       </c>
       <c r="W422" t="inlineStr">
         <is>
-          <t>[35.0, 18.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -31335,7 +31335,7 @@
       </c>
       <c r="W423" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -31408,7 +31408,7 @@
       </c>
       <c r="W424" t="inlineStr">
         <is>
-          <t>[37.5, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -31700,7 +31700,7 @@
       </c>
       <c r="W428" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31773,7 +31773,7 @@
       </c>
       <c r="W429" t="inlineStr">
         <is>
-          <t>[27.5, 24.0, 320.0]</t>
+          <t>[30.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31846,7 +31846,7 @@
       </c>
       <c r="W430" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -31919,7 +31919,7 @@
       </c>
       <c r="W431" t="inlineStr">
         <is>
-          <t>[25.0, 20.0, 320.0]</t>
+          <t>[27.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -31992,7 +31992,7 @@
       </c>
       <c r="W432" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 320.0]</t>
+          <t>[30.0, 14.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32065,7 +32065,7 @@
       </c>
       <c r="W433" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -32138,7 +32138,7 @@
       </c>
       <c r="W434" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 355.0]</t>
+          <t>[30.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -32211,7 +32211,7 @@
       </c>
       <c r="W435" t="inlineStr">
         <is>
-          <t>[25.0, 22.0, 320.0]</t>
+          <t>[25.0, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32357,7 +32357,7 @@
       </c>
       <c r="W437" t="inlineStr">
         <is>
-          <t>[35.0, 22.0, 400.0]</t>
+          <t>[35.0, 20.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -32503,7 +32503,7 @@
       </c>
       <c r="W439" t="inlineStr">
         <is>
-          <t>[25.0, 18.0, 320.0]</t>
+          <t>[25.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -32576,7 +32576,7 @@
       </c>
       <c r="W440" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -32649,7 +32649,7 @@
       </c>
       <c r="W441" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 355.0]</t>
+          <t>[35.0, 14.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -32722,7 +32722,7 @@
       </c>
       <c r="W442" t="inlineStr">
         <is>
-          <t>[30.0, 18.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -32795,7 +32795,7 @@
       </c>
       <c r="W443" t="inlineStr">
         <is>
-          <t>[27.5, 20.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -32868,7 +32868,7 @@
       </c>
       <c r="W444" t="inlineStr">
         <is>
-          <t>[25.0, 16.0, 320.0]</t>
+          <t>[27.5, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33014,7 +33014,7 @@
       </c>
       <c r="W446" t="inlineStr">
         <is>
-          <t>[30.0, 20.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33087,7 +33087,7 @@
       </c>
       <c r="W447" t="inlineStr">
         <is>
-          <t>[27.5, 14.0, 345.0]</t>
+          <t>[30.0, 14.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33160,7 +33160,7 @@
       </c>
       <c r="W448" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 360.0]</t>
+          <t>[32.5, 16.0, 360.0]</t>
         </is>
       </c>
     </row>
@@ -33306,7 +33306,7 @@
       </c>
       <c r="W450" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33379,7 +33379,7 @@
       </c>
       <c r="W451" t="inlineStr">
         <is>
-          <t>[30.0, 16.0, 370.0]</t>
+          <t>[32.5, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33452,7 +33452,7 @@
       </c>
       <c r="W452" t="inlineStr">
         <is>
-          <t>[30.0, 12.0, 370.0]</t>
+          <t>[32.5, 12.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33598,7 +33598,7 @@
       </c>
       <c r="W454" t="inlineStr">
         <is>
-          <t>[27.5, 22.0, 345.0]</t>
+          <t>[30.0, 20.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33671,7 +33671,7 @@
       </c>
       <c r="W455" t="inlineStr">
         <is>
-          <t>[40.0, 16.0, 370.0]</t>
+          <t>[35.0, 16.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -33744,7 +33744,7 @@
       </c>
       <c r="W456" t="inlineStr">
         <is>
-          <t>[37.5, 20.0, 355.0]</t>
+          <t>[35.0, 20.0, 355.0]</t>
         </is>
       </c>
     </row>
@@ -33817,7 +33817,7 @@
       </c>
       <c r="W457" t="inlineStr">
         <is>
-          <t>[27.5, 16.0, 320.0]</t>
+          <t>[30.0, 16.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -33890,7 +33890,7 @@
       </c>
       <c r="W458" t="inlineStr">
         <is>
-          <t>[27.5, 18.0, 345.0]</t>
+          <t>[30.0, 16.0, 345.0]</t>
         </is>
       </c>
     </row>
@@ -33963,7 +33963,7 @@
       </c>
       <c r="W459" t="inlineStr">
         <is>
-          <t>[35.0, 18.0, 400.0]</t>
+          <t>[35.0, 16.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34036,7 +34036,7 @@
       </c>
       <c r="W460" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 370.0]</t>
+          <t>[32.5, 14.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -34255,7 +34255,7 @@
       </c>
       <c r="W463" t="inlineStr">
         <is>
-          <t>[25.0, 24.0, 320.0]</t>
+          <t>[27.5, 20.0, 320.0]</t>
         </is>
       </c>
     </row>
@@ -34401,7 +34401,7 @@
       </c>
       <c r="W465" t="inlineStr">
         <is>
-          <t>[37.5, 14.0, 400.0]</t>
+          <t>[35.0, 14.0, 400.0]</t>
         </is>
       </c>
     </row>
@@ -34547,7 +34547,7 @@
       </c>
       <c r="W467" t="inlineStr">
         <is>
-          <t>[30.0, 22.0, 370.0]</t>
+          <t>[32.5, 20.0, 370.0]</t>
         </is>
       </c>
     </row>
@@ -34620,7 +34620,7 @@
       </c>
       <c r="W468" t="inlineStr">
         <is>
-          <t>[40.0, 16.0, 390.0]</t>
+          <t>[35.0, 16.0, 390.0]</t>
         </is>
       </c>
     </row>
@@ -34693,7 +34693,7 @@
       </c>
       <c r="W469" t="inlineStr">
         <is>
-          <t>[30.0, 14.0, 360.0]</t>
+          <t>[32.5, 14.0, 360.0]</t>
         </is>
       </c>
     </row>

</xml_diff>